<commit_message>
Updated example system threat modeling workbook to add missing ESD-10 source authentication information
</commit_message>
<xml_diff>
--- a/source/reference_documents/working_material/example system/example system threat model r2.xlsx
+++ b/source/reference_documents/working_material/example system/example system threat model r2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/example system/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1153CB-0ABB-F548-8E1A-1C81885E503D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BB0F8F-0BAE-9A4D-97D6-081E3ABD6378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16920" yWindow="12880" windowWidth="33760" windowHeight="20720" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="294">
   <si>
     <t>DO NOT EDIT THIS PAGE</t>
   </si>
@@ -1204,23 +1204,23 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1228,20 +1228,20 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1585,18 +1585,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="59">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
     </row>
     <row r="3" spans="2:11">
       <c r="B3" s="13"/>
@@ -1611,10 +1611,10 @@
       <c r="K3" s="13"/>
     </row>
     <row r="4" spans="2:11" ht="30">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="33"/>
+      <c r="C4" s="29"/>
       <c r="D4" s="34" t="s">
         <v>81</v>
       </c>
@@ -1627,22 +1627,22 @@
       <c r="K4" s="13"/>
     </row>
     <row r="5" spans="2:11">
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
       <c r="K5" s="13"/>
     </row>
     <row r="6" spans="2:11" ht="30">
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="33"/>
+      <c r="C6" s="29"/>
       <c r="D6" s="34" t="s">
         <v>82</v>
       </c>
@@ -1655,78 +1655,78 @@
       <c r="K6" s="13"/>
     </row>
     <row r="7" spans="2:11">
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
       <c r="K7" s="13"/>
     </row>
     <row r="8" spans="2:11" ht="30">
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="37" t="s">
+      <c r="C8" s="29"/>
+      <c r="D8" s="36" t="s">
         <v>83</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="37"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="36"/>
       <c r="K8" s="13"/>
     </row>
     <row r="9" spans="2:11">
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
       <c r="K9" s="13"/>
     </row>
     <row r="10" spans="2:11" ht="30">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="37" t="s">
+      <c r="C10" s="29"/>
+      <c r="D10" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
       <c r="K10" s="13"/>
     </row>
     <row r="11" spans="2:11">
-      <c r="B11" s="36"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
       <c r="K11" s="13"/>
     </row>
     <row r="12" spans="2:11" ht="30">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="33"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="38" t="s">
         <v>22</v>
       </c>
@@ -1739,59 +1739,59 @@
       <c r="K12" s="13"/>
     </row>
     <row r="13" spans="2:11">
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="36"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
       <c r="K13" s="13"/>
     </row>
     <row r="14" spans="2:11" ht="30">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="39">
+      <c r="C14" s="29"/>
+      <c r="D14" s="37">
         <v>45715</v>
       </c>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="37"/>
       <c r="K14" s="13"/>
     </row>
     <row r="15" spans="2:11">
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
       <c r="K15" s="13"/>
     </row>
     <row r="16" spans="2:11" ht="30">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="40">
+      <c r="C16" s="29"/>
+      <c r="D16" s="31">
         <v>2</v>
       </c>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="36"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="36"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
       <c r="K16" s="13"/>
     </row>
     <row r="17" spans="2:11" ht="134" customHeight="1">
@@ -1807,18 +1807,18 @@
       <c r="K17" s="13"/>
     </row>
     <row r="18" spans="2:11" ht="28">
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="29"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1861,22 +1861,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="39"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -2292,7 +2292,9 @@
       <c r="I14" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="J14" s="21"/>
+      <c r="J14" s="21" t="s">
+        <v>39</v>
+      </c>
       <c r="K14" s="21"/>
       <c r="L14" s="21"/>
       <c r="M14" s="21" t="s">
@@ -4640,11 +4642,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -4777,11 +4779,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -4898,17 +4900,17 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="2" spans="2:10" ht="59">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="13"/>
@@ -4933,17 +4935,17 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="2:10" ht="25">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
     </row>
     <row r="7" spans="2:10" ht="17">
       <c r="B7" t="s">
@@ -4966,17 +4968,17 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="2" spans="2:10" ht="59">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="13"/>
@@ -5001,17 +5003,17 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" spans="2:10" ht="25">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5041,20 +5043,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -5490,17 +5492,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:14" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -5960,13 +5962,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -6150,13 +6152,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="63">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>

</xml_diff>